<commit_message>
fix para consolidacion "novedades" y "asignaciones" nextfocus: incluir en curva Real los turnos de "Novedades"
</commit_message>
<xml_diff>
--- a/Result/AsignacionTurnos.xlsx
+++ b/Result/AsignacionTurnos.xlsx
@@ -429,12 +429,12 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Inicio</t>
+          <t>Hora_Inicio</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Fin</t>
+          <t>Hora_Termino</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">

</xml_diff>